<commit_message>
Belge arşivi: coğrafya yıllık planları 2026.08.1 — çizelge ve açıklamalar ayrı çalışma sayfalarına ayrıldı (yinelenen başlık ilgisiz bölümlere taşmıyor)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/evrak/cografya-yillik-planlari/GNL-CYP-CP-001_Cografya_9_Sinif_Yillik_Plani_v1.0.xlsx
+++ b/public/evrak/cografya-yillik-planlari/GNL-CYP-CP-001_Cografya_9_Sinif_Yillik_Plani_v1.0.xlsx
@@ -8,9 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9.SINIF" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Açıklamalar ve Onay" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'9.SINIF'!$1:$2</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Açıklamalar ve Onay'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -543,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H108"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.3" customWidth="1" min="1" max="1"/>
@@ -1765,32 +1767,759 @@
       <c r="G44" s="5" t="n"/>
       <c r="H44" s="5" t="n"/>
     </row>
-    <row r="46" ht="14" customHeight="1">
-      <c r="A46" s="11" t="inlineStr">
+  </sheetData>
+  <mergeCells count="41">
+    <mergeCell ref="A36:A39"/>
+    <mergeCell ref="E14:E17"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="D24:D26"/>
+    <mergeCell ref="D21:H21"/>
+    <mergeCell ref="A19:A21"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="G37:G38"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="G24:G25"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A40:A42"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="F6:F8"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A32:A35"/>
+    <mergeCell ref="D33:D34"/>
+    <mergeCell ref="G14:G17"/>
+    <mergeCell ref="A23:A26"/>
+    <mergeCell ref="G33:G34"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="D6:D10"/>
+    <mergeCell ref="F37:F38"/>
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="E6:E8"/>
+    <mergeCell ref="A6:A10"/>
+    <mergeCell ref="D14:D17"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="F14:F17"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D35:D38"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="A28:A31"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="D3:D5"/>
+    <mergeCell ref="G6:G8"/>
+    <mergeCell ref="A15:A18"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="F24:F25"/>
+  </mergeCells>
+  <pageMargins left="0.39" right="0.39" top="0.55" bottom="0.55" header="0.25" footer="0.25"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;LGNL-CYP-CP-001 · okulapp.org&amp;RSayfa &amp;P / &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:H65"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5.3" customWidth="1" min="1" max="1"/>
+    <col width="9.01" customWidth="1" min="2" max="2"/>
+    <col width="4.77" customWidth="1" min="3" max="3"/>
+    <col width="10.6" customWidth="1" min="4" max="4"/>
+    <col width="13.78" customWidth="1" min="5" max="5"/>
+    <col width="29.68" customWidth="1" min="6" max="6"/>
+    <col width="50.88" customWidth="1" min="7" max="7"/>
+    <col width="13.25" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="00C00000"/>
+              <sz val="11"/>
+            </rPr>
+            <t>[OKUL ADI]</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> 2026-2027 EĞİTİM ÖĞRETİM YILI 9. SINIF COĞRAFYA DERSİ YILLIK PLANI — AÇIKLAMALAR VE ONAY</t>
+          </r>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+    </row>
+    <row r="3" ht="14" customHeight="1">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>ÖĞRENME KANITLARI (ÖLÇME VE DEĞERLENDİRME) — ünite/hafta bazında</t>
         </is>
       </c>
-      <c r="B46" s="12" t="n"/>
-      <c r="C46" s="12" t="n"/>
-      <c r="D46" s="12" t="n"/>
-      <c r="E46" s="12" t="n"/>
-      <c r="F46" s="12" t="n"/>
-      <c r="G46" s="12" t="n"/>
-      <c r="H46" s="12" t="n"/>
-    </row>
-    <row r="47" ht="45.4" customHeight="1">
-      <c r="A47" s="4" t="inlineStr">
+      <c r="B3" s="12" t="n"/>
+      <c r="C3" s="12" t="n"/>
+      <c r="D3" s="12" t="n"/>
+      <c r="E3" s="12" t="n"/>
+      <c r="F3" s="12" t="n"/>
+      <c r="G3" s="12" t="n"/>
+      <c r="H3" s="12" t="n"/>
+    </row>
+    <row r="4" ht="45.4" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>1-3. haftalar</t>
         </is>
       </c>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Öğrenme çıktıları; zihin haritası, Frayer diyagramı, açık uçlu sorular, öz değerlendirme formu, performans görevi, analitik dereceli puanlama anahtarı, grup değerlendirme formu kullanılarak değerlendirilebilir. Performans görevi olarak öğrencilerden örnek olay, olgu veya konu üzerinden mekânsal düşünme ile coğrafya öğrenmenin önemini ortaya koyan bir gazete haberi yazmaları istenebilir. Performans görevi; bilgi toplama, bilgileri düzenlenme, haber oluşturma ve sunum yapma ölçütlerine göre değerlendirilebilir.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+    </row>
+    <row r="5" ht="45.4" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>4-8. haftalar</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Öğrenme çıktıları; kontrol listesi, çalışma yaprağı, anlam çözümleme tablosu, performans görevi, analitik dereceli puanlama anahtarı, öz değerlendirme formu ve grup değerlendirme formu kullanılarak değerlendirilebilir. Performans görevi olarak öğrencilerden dilsiz harita üzerinde belirli bir konu içeriğine sahip harita oluşturmaları istenebilir. Performans görevi; amaç belirleme, araç gereç seçme ve kullanma, veri toplama, toplanan verileri seçme ve işleme, sembol belirleme, harita bileşenlerini oluşturma ölçütlerine göre değerlendirilebilir.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
+    </row>
+    <row r="6" ht="45.4" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>9. hafta</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Öğrenme çıktıları; çalışma yaprağı, açık uçlu sorular, kontrol listesi, öğrenme günlüğü, performans görevi, analitik dereceli puanlama anahtarı, öz değerlendirme formu ve grup değerlendirme formu kullanılarak değerlendirilebilir. Performans görevi olarak öğrencilerden farklı iklim türlerine sahip yerlerdeki küresel iklim değişikliğinin yansımalarına ilişkin bilgi görseli hazırlamaları istenebilir. Performans göre-vi; amaç belirleme, bilgi toplama, bilgileri düzenlenme ve görselleştirme, sunum yapma ölçütlerine göre değerlendirilebilir.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+    </row>
+    <row r="7" ht="45.4" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>10-15. haftalar, 16-17. haftalar, 19. hafta</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Öğrenme çıktıları; çalışma yaprağı, açık uçlu sorular, kontrol listesi, öğrenme günlüğü, performans görevi, analitik dereceli puanlama anahtarı, öz değerlendirme formu ve grup değerlendirme formu kullanılarak değerlendirilebilir. Performans görevi olarak öğrencilerden farklı iklim türlerine sahip yerlerdeki küresel iklim değişikliğinin yansımalarına ilişkin bilgi görseli hazırlamaları istenebilir. Performans görevi; amaç belirleme, bilgi toplama, bilgileri düzenlenme ve görselleştirme, sunum yapma ölçütlerine göre değerlendirilebilir.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+    </row>
+    <row r="8" ht="45.4" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>20-22. haftalar, 23-26. haftalar, 27. hafta</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Öğrenme çıktıları; çalışma yaprağı, açık uçlu sorular, öğrenme günlüğü, performans gö-revi, analitik dereceli puanlama anahtarı, öz değerlendirme formu, grup değerlendirme formu kullanılarak değerlendirilebilir. Performans görevi olarak öğrencilerden grup etkinliği şeklinde Türkiye nüfusundaki değişim seyrinin nüfusla ilgili fırsat, sorun ve politikalara etkisini belirlemek amacıyla araş-tırma yapmaları ve bu araştırmayı raporlaştırmaları istenebilir. Performans görevi; hazırlık yapma, bilgi toplama, bilgileri çözümleme ve rapor yazma ölçütlerine göre değerlendirilebilir.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
+    </row>
+    <row r="9" ht="45.4" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>28-29. haftalar</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Öğrenme çıktısı; KWL (ne biliyorum-ne bilmek istiyorum-ne öğrendim), performans gö-revi, analitik dereceli puanlama anahtarı, öz değerlendirme formu kullanılarak değerlendirilebilir. Performans görevi olarak öğrencilerden doğal ve beşerî faktörlerin ekonomi üzerindeki etkilerini harita, fotoğraf vb. görsellerle açıklayan bir diyagram hazırlamaları istenebilir. Performans görevi; bilgi toplama, bilgileri düzenleme, görsel materyal kullanma ve diyagram hazırlama ölçütlerine göre değerlendirilebilir.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+    </row>
+    <row r="10" ht="45.4" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>30-33. haftalar</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Öğrenme çıktıları; çalışma yaprağı, yapılandırılmış grid, performans görevi, analitik dere-celi puanlama anahtarı, öz değerlendirme formu kullanılarak değerlendirilebilir. Performans görevi olarak öğrencilerden örnek bir senaryo üzerinden bütüncül afet yönetimine ilişkin önerilerini içeren bir sunum hazırlamaları istenebilir. Performans görevi; bilgi inceleme, içerik, sonuç çıkarma, rapor hazırlama ve sunma ölçütlerine göre değerlendirilebilir.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
+    </row>
+    <row r="11" ht="45.4" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>34. hafta, 35. hafta</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Öğrenme çıktısı; anlam çözümleme tablosu, açık uçlu sorular, performans görevi, analitik dereceli puanlama anahtarı, öz değerlendirme formu, grup değerlendirme formu kullanılarak değerlendirilebilir. Performans görevi olarak öğrenci gruplarından farklı haritalar üzerinde bölge belirleme kriterlerini dikkate alarak bölgeler oluşturmaları istenebilir. Performans görevi; harita seçme, karşılaştırma yapma, önermede bulunma, sonuç çıkarma, bölge belirleme ve sunma ölçütlerine göre değerlendirilebilir.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+    </row>
+    <row r="13" ht="14" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>SOSYAL - DUYGUSAL ÖĞRENME BECERİLERİ — ünite/hafta bazında</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="n"/>
+      <c r="C13" s="12" t="n"/>
+      <c r="D13" s="12" t="n"/>
+      <c r="E13" s="12" t="n"/>
+      <c r="F13" s="12" t="n"/>
+      <c r="G13" s="12" t="n"/>
+      <c r="H13" s="12" t="n"/>
+    </row>
+    <row r="14" ht="24.2" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>1-3. haftalar</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>SDB1.1. Kendini Tanıma (Öz Farkındalık), SDB1.2. Kendini Düzenleme (Öz Düzenleme), SDB1.3. Kendine Uyarlama (Öz Yansıtma), SDB2.1. İletişim, SDB2.2. İş Birliği, SDB2.3. Sos-yal Farkındalık</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
+    </row>
+    <row r="15" ht="24.2" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>4-8. haftalar, 28-29. haftalar</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>SDB1.1. Kendini Tanıma (Öz Farkındalık), SDB1.2. Kendini Düzenleme (Öz Düzenleme), SDB1.3. Kendine Uyarlama (Öz Yansıtma), SDB2.1. İletişim, SDB2.2. İş Birliği</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
+    </row>
+    <row r="16" ht="45.4" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>9. hafta, 10-15. haftalar, 16-17. haftalar, 19. hafta</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>SDB1.1. Kendini Tanıma (Öz Farkındalık), SDB1.2. Kendini Düzenleme (Öz Düzenleme), SDB2.1. İletişim, SDB2.2. İş Birliği, SDB2.3. Sosyal Farkındalık, SDB3.3. Sorumlu Karar Verme</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+    </row>
+    <row r="17" ht="34.8" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>20-22. haftalar, 23-26. haftalar, 27. hafta</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>SDB1.1. Kendini Tanıma (Öz Farkındalık), SDB1.2. Kendini Düzenleme (Öz Düzenleme), SDB1.3. Kendine Uyarlama (Öz Yansıtma), SDB2.1. İletişim, SDB2.2. İş Birliği, SDB3.3. Sorumlu Karar Verme</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+    </row>
+    <row r="18" ht="24.2" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>30-33. haftalar</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>DB1.1. Kendini Tanıma (Öz Farkındalık), SDB1.2. Kendini Düzenleme (Öz Düzenleme), SDB1.3. Kendine Uyarlama (Öz Yansıtma), SDB2.1. İletişim, SDB2.2. İş Birliği, SDB2.3. Sos-yal Farkındalık, SDB3.3. Sorumlu Karar Verme</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
+    </row>
+    <row r="19" ht="24.2" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>34. hafta, 35. hafta</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>SDB1.2. Kendini Düzenleme (Öz Düzenleme), SDB1.3. Kendine Uyarlama (Öz Yansıtma), DB2.1. İletişim, SDB2.2. İş Birliği</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
+    </row>
+    <row r="21" ht="14" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>DEĞERLER — ünite/hafta bazında</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="n"/>
+      <c r="C21" s="12" t="n"/>
+      <c r="D21" s="12" t="n"/>
+      <c r="E21" s="12" t="n"/>
+      <c r="F21" s="12" t="n"/>
+      <c r="G21" s="12" t="n"/>
+      <c r="H21" s="12" t="n"/>
+    </row>
+    <row r="22" ht="13.6" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>1-3. haftalar</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>D3. Çalışkanlık, D14. Saygı, D16. Sorumluluk, D19. Vatanseverlik</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+    </row>
+    <row r="23" ht="13.6" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>4-8. haftalar</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>D3. Çalışkanlık, D10. Mütevazılık, D11. Özgürlük, D19. Vatanseverlik</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+    </row>
+    <row r="24" ht="45.4" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>9. hafta, 10-15. haftalar, 16-17. haftalar, 19. hafta</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n"/>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>D3. Çalışkanlık, D5. Duyarlılık, D9. Merhamet, D14. Saygı</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
+    </row>
+    <row r="25" ht="24.2" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>20-22. haftalar, 23-26. haftalar</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>D2. Aile Bütünlüğü, D3. Çalışkanlık, D4. Dostluk, D14. Saygı</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n"/>
+    </row>
+    <row r="26" ht="13.6" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>27. hafta</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>D2. Aile Bütünlüğü, D3. Çalışkanlık, D4. Dostluk, D14. Sayg</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
+    </row>
+    <row r="27" ht="13.6" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>28-29. haftalar</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n"/>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>D17. Tasarruf, D19. Vatanseverlik</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="n"/>
+    </row>
+    <row r="28" ht="13.6" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>30-33. haftalar</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>D1. Adalet, D5. Duyarlılık, D16. Sorumluluk, D20. Yardımseverlik</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="n"/>
+    </row>
+    <row r="29" ht="24.2" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>34. hafta, 35. hafta</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>D3. Çalışkanlık</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="n"/>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="n"/>
+      <c r="H29" s="2" t="n"/>
+    </row>
+    <row r="31" ht="14" customHeight="1">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>OKURYAZARLIK BECERİLERİ — ünite/hafta bazında</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="n"/>
+      <c r="C31" s="12" t="n"/>
+      <c r="D31" s="12" t="n"/>
+      <c r="E31" s="12" t="n"/>
+      <c r="F31" s="12" t="n"/>
+      <c r="G31" s="12" t="n"/>
+      <c r="H31" s="12" t="n"/>
+    </row>
+    <row r="32" ht="13.6" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>1-3. haftalar</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>OB1. Bilgi Okuryazarlığı, OB4. Görsel Okuryazarlık</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="n"/>
+    </row>
+    <row r="33" ht="24.2" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>4-8. haftalar, 30-33. haftalar</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>OB1. Bilgi Okuryazarlığı, OB2. Dijital Okuryazarlık, OB4. Görsel Okuryazarlık</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2" t="n"/>
+      <c r="H33" s="2" t="n"/>
+    </row>
+    <row r="34" ht="45.4" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>9. hafta, 10-15. haftalar, 16-17. haftalar, 19. hafta</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>OB2. Dijital Okuryazarlık, OB4. Görsel Okuryazarlık, OB5. Kültür Okuryazarlığı, OB7. Veri Okuryazarlığı, OB8. Sürdürülebilirlik Okuryazarlığı</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="n"/>
+    </row>
+    <row r="35" ht="34.8" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>20-22. haftalar, 23-26. haftalar, 27. hafta</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>OB1. Bilgi Okuryazarlığı, OB4. Görsel Okuryazarlık, OB7. Veri Okuryazarlığı</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="n"/>
+      <c r="H35" s="2" t="n"/>
+    </row>
+    <row r="36" ht="13.6" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>28-29. haftalar</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>OB1. Bilgi Okuryazarlığı</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2" t="n"/>
+      <c r="H36" s="2" t="n"/>
+    </row>
+    <row r="37" ht="24.2" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>34. hafta, 35. hafta</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>OB2. Dijital Okuryazarlık</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2" t="n"/>
+      <c r="H37" s="2" t="n"/>
+    </row>
+    <row r="39" ht="14" customHeight="1">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>FARKLILAŞTIRMA</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="n"/>
+      <c r="C39" s="12" t="n"/>
+      <c r="D39" s="12" t="n"/>
+      <c r="E39" s="12" t="n"/>
+      <c r="F39" s="12" t="n"/>
+      <c r="G39" s="12" t="n"/>
+      <c r="H39" s="12" t="n"/>
+    </row>
+    <row r="40" ht="45.4" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Türkiye Yüzyılı Maarif Modeli Ortak Metni'nde “Farklılaştırılmış öğrenme yaşantılarında öğrencilerin ilgi alanları ile öğrenme profilleri önemlidir ve öğrencilere çeşitli öğrenme yaşantıları sunulur. Farklılaştırma kapsamında yapılacak zenginleştirme ve destekleme uygulamalarında öğrencilerin bireysel farklılıkları (öğrenme hızları, öğrenme stilleri, yetenekleri vb.), ilgi ve ihtiyaçları dikkate alınarak gereken planlamalar yapılır.” ifadesi yer almaktadır. Öğretmenler sınıftaki öğrencilerini gözlemleyerek gerek gördükleri konularda farklılaştırma uygulamalarını ders sürecine dâhil etmelidirler.</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="2" t="n"/>
+      <c r="H40" s="2" t="n"/>
+    </row>
+    <row r="42" ht="14" customHeight="1">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>OKUL TEMELLİ PLANLAMA — ÇERÇEVE PLAN AÇIKLAMASI</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="n"/>
+      <c r="C42" s="12" t="n"/>
+      <c r="D42" s="12" t="n"/>
+      <c r="E42" s="12" t="n"/>
+      <c r="F42" s="12" t="n"/>
+      <c r="G42" s="12" t="n"/>
+      <c r="H42" s="12" t="n"/>
+    </row>
+    <row r="43" ht="119.6" customHeight="1">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Okul temelli planlama; zümre öğretmenler kurulu tarafından ders kapsamında gerçekleştirilmesi kararlaştırılan araştırma ve gözlem, sosyal etkinlikler, proje çalışmaları, yerel çalışmalar, okuma çalışmaları vb. çalışmaları kapsamaktadır. Çalışmalar için ayrılan süre eğitim-öğretim yılı içinde planlanır ve yıllık planlarda ifade edilir. Bu planlamalar kapsamında yürütülecek öğretim faaliyetleri; öğrenci katılımını desteklemeli, yaparak ve yaşayarak öğrenmeye olanak tanımalı, öğrencinin bütüncül gelişime hizmet etmelidir. *Bu çerçeve planda belirtilen okul temelli planlama haftaları örnek olarak sunulmuştur. Zümre öğretmenler kurulunda aldığınız karara göre okul ve ders koşullarınıza uygun (öğretim programında belirtilen okul temelli planlama ders saati 2 haftadan fazla sürebilir) düzenleyebilirsiniz.Okul temelli planlama; zümre öğretmenler kurulu tarafından ders kapsamında gerçekleştirilmesi kararlaştırılan araştırma ve gözlem, sosyal etkinlikler, proje çalışmaları, yerel çalışmalar, okuma çalışmaları vb. çalışmaları kapsamaktadır. Çalışmalar için ayrılan süre eğitim-öğretim yılı içinde planlanır ve yıllık planlarda ifade edilir. Bu planlamalar kapsamında yürütülecek öğretim faaliyetleri; öğrenci katılımını desteklemeli, yaparak ve yaşayarak öğrenmeye olanak tanımalı, öğrencinin bütüncül gelişime hizmet etmelidir. *Bu çerçeve planda belirtilen okul temelli planlama haftaları örnek olarak sunulmuştur. Zümre öğretmenler kurulunda aldığınız karara göre okul ve ders koşullarınıza uygun (öğretim programında belirtilen okul temelli planlama ders saati 2 haftadan fazla sürebilir) düzenleyebilirsiniz.</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
+      <c r="G43" s="2" t="n"/>
+      <c r="H43" s="2" t="n"/>
+    </row>
+    <row r="45" ht="14" customHeight="1">
+      <c r="A45" s="11" t="inlineStr">
+        <is>
+          <t>OKUL UYARLAMA NOTLARI</t>
+        </is>
+      </c>
+      <c r="B45" s="12" t="n"/>
+      <c r="C45" s="12" t="n"/>
+      <c r="D45" s="12" t="n"/>
+      <c r="E45" s="12" t="n"/>
+      <c r="F45" s="12" t="n"/>
+      <c r="G45" s="12" t="n"/>
+      <c r="H45" s="12" t="n"/>
+    </row>
+    <row r="46" ht="24.2" customHeight="1">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>GENEL ŞABLON: Bu plan, okulapp.org belge arşivinde yayımlanan genel sürümdür (CC BY 4.0). Köşeli parantezli KIRMIZI alanlar (okul adı, ad-soyad, tarih) okulun bilgileriyle doldurulur; doldurduktan sonra parantez kaldırılır ve yazı rengi siyaha çevrilir.</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="n"/>
+      <c r="C46" s="2" t="n"/>
+      <c r="D46" s="2" t="n"/>
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="n"/>
+      <c r="G46" s="2" t="n"/>
+      <c r="H46" s="2" t="n"/>
+    </row>
+    <row r="47" ht="34.8" customHeight="1">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>KAYNAK: Bu plan, Millî Eğitim Bakanlığının tymm.meb.gov.tr/taslak-cerceve-planlari adresinde yayımladığı 2026-2027 eğitim öğretim yılı Anadolu lisesi coğrafya dersi taslak çerçeve yıllık planının "9.SINIF" sayfasından, içeriği değiştirilmeden A4 yatay sayfaya yeniden yerleştirilerek okula uyarlanmıştır (erişim 29.08.2026). Ünite bazlı öğrenme kanıtları ile programlar arası bileşenler, okunabilirlik için haftalık çizelgenin altındaki bölümlere taşınmıştır.</t>
+        </is>
+      </c>
       <c r="B47" s="2" t="n"/>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>Öğrenme çıktıları; zihin haritası, Frayer diyagramı, açık uçlu sorular, öz değerlendirme formu, performans görevi, analitik dereceli puanlama anahtarı, grup değerlendirme formu kullanılarak değerlendirilebilir. Performans görevi olarak öğrencilerden örnek olay, olgu veya konu üzerinden mekânsal düşünme ile coğrafya öğrenmenin önemini ortaya koyan bir gazete haberi yazmaları istenebilir. Performans görevi; bilgi toplama, bilgileri düzenlenme, haber oluşturma ve sunum yapma ölçütlerine göre değerlendirilebilir.</t>
-        </is>
-      </c>
+      <c r="C47" s="2" t="n"/>
       <c r="D47" s="2" t="n"/>
       <c r="E47" s="2" t="n"/>
       <c r="F47" s="2" t="n"/>
@@ -1798,689 +2527,63 @@
       <c r="H47" s="2" t="n"/>
     </row>
     <row r="48" ht="45.4" customHeight="1">
-      <c r="A48" s="4" t="inlineStr">
-        <is>
-          <t>4-8. haftalar</t>
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>ÇALIŞMA TAKVİMİ UYARLAMASI (il millî eğitim müdürlüğü 2026-2027 çalışma takvimi — tarihler Bakanlık takvimiyle ortaktır, ilinizin takvimini kontrol ediniz): Kurban Bayramı tatili 15-19 Mayıs 2027 olup planın 32. haftasına denk gelir; o hafta yalnız perşembe ve cuma günleri ders yapılır ve 19 Mayıs Atatürk'ü Anma, Gençlik ve Spor Bayramı bayram tatili içinde kalır. 28 Ekim 2026 çarşamba yarım gündür; 1 Ocak 2027 cuma ile 23 Nisan 2027 cuma resmî tatildir. Bu günlere gelen ders saatlerinde konu akışı zümre kararıyla yoğunlaştırılarak telafi edilir.</t>
         </is>
       </c>
       <c r="B48" s="2" t="n"/>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>Öğrenme çıktıları; kontrol listesi, çalışma yaprağı, anlam çözümleme tablosu, performans görevi, analitik dereceli puanlama anahtarı, öz değerlendirme formu ve grup değerlendirme formu kullanılarak değerlendirilebilir. Performans görevi olarak öğrencilerden dilsiz harita üzerinde belirli bir konu içeriğine sahip harita oluşturmaları istenebilir. Performans görevi; amaç belirleme, araç gereç seçme ve kullanma, veri toplama, toplanan verileri seçme ve işleme, sembol belirleme, harita bileşenlerini oluşturma ölçütlerine göre değerlendirilebilir.</t>
-        </is>
-      </c>
+      <c r="C48" s="2" t="n"/>
       <c r="D48" s="2" t="n"/>
       <c r="E48" s="2" t="n"/>
       <c r="F48" s="2" t="n"/>
       <c r="G48" s="2" t="n"/>
       <c r="H48" s="2" t="n"/>
     </row>
-    <row r="49" ht="45.4" customHeight="1">
-      <c r="A49" s="4" t="inlineStr">
-        <is>
-          <t>9. hafta</t>
+    <row r="49" ht="34.8" customHeight="1">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>OKUL TEMELLİ PLANLAMA: Çizelgedeki kırmızı ekler zümre karar taslağıdır; sene başı zümre toplantısında kesinleştirilir, kesinleşen kullanım bu satırlara işlenerek kırmızı ibare siyaha çevrilir. Çerçeve plandaki 18. ve 36. hafta yerleşimi örnektir; zümre kararıyla değiştirilebilir. Öğrenme kanıtları zümre dosyasında toplanır; okul dışına çıkılan çalışmalarda zaman-yer-refakat onayı ile veli izni okulun sosyal etkinlik belgeleri üzerinden alınır.</t>
         </is>
       </c>
       <c r="B49" s="2" t="n"/>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>Öğrenme çıktıları; çalışma yaprağı, açık uçlu sorular, kontrol listesi, öğrenme günlüğü, performans görevi, analitik dereceli puanlama anahtarı, öz değerlendirme formu ve grup değerlendirme formu kullanılarak değerlendirilebilir. Performans görevi olarak öğrencilerden farklı iklim türlerine sahip yerlerdeki küresel iklim değişikliğinin yansımalarına ilişkin bilgi görseli hazırlamaları istenebilir. Performans göre-vi; amaç belirleme, bilgi toplama, bilgileri düzenlenme ve görselleştirme, sunum yapma ölçütlerine göre değerlendirilebilir.</t>
-        </is>
-      </c>
+      <c r="C49" s="2" t="n"/>
       <c r="D49" s="2" t="n"/>
       <c r="E49" s="2" t="n"/>
       <c r="F49" s="2" t="n"/>
       <c r="G49" s="2" t="n"/>
       <c r="H49" s="2" t="n"/>
     </row>
-    <row r="50" ht="45.4" customHeight="1">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>10-15. haftalar, 16-17. haftalar, 19. hafta</t>
+    <row r="50" ht="13.6" customHeight="1">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>ÖLÇME VE DEĞERLENDİRME: Yazılı sınav tarihleri bu planda gösterilmez; okul sınav takvimi ve zümrenin ortak sınav planlamasına göre yürütülür.</t>
         </is>
       </c>
       <c r="B50" s="2" t="n"/>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>Öğrenme çıktıları; çalışma yaprağı, açık uçlu sorular, kontrol listesi, öğrenme günlüğü, performans görevi, analitik dereceli puanlama anahtarı, öz değerlendirme formu ve grup değerlendirme formu kullanılarak değerlendirilebilir. Performans görevi olarak öğrencilerden farklı iklim türlerine sahip yerlerdeki küresel iklim değişikliğinin yansımalarına ilişkin bilgi görseli hazırlamaları istenebilir. Performans görevi; amaç belirleme, bilgi toplama, bilgileri düzenlenme ve görselleştirme, sunum yapma ölçütlerine göre değerlendirilebilir.</t>
-        </is>
-      </c>
+      <c r="C50" s="2" t="n"/>
       <c r="D50" s="2" t="n"/>
       <c r="E50" s="2" t="n"/>
       <c r="F50" s="2" t="n"/>
       <c r="G50" s="2" t="n"/>
       <c r="H50" s="2" t="n"/>
     </row>
-    <row r="51" ht="45.4" customHeight="1">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>20-22. haftalar, 23-26. haftalar, 27. hafta</t>
+    <row r="51" ht="13.6" customHeight="1">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>ATATÜRKÇÜLÜK KONULARI: 2488 sayılı Tebliğler Dergisi'ndeki Atatürkçülük konuları, zümre kararı doğrultusunda ilgili ünitelere dağıtılarak işlenir.</t>
         </is>
       </c>
       <c r="B51" s="2" t="n"/>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>Öğrenme çıktıları; çalışma yaprağı, açık uçlu sorular, öğrenme günlüğü, performans gö-revi, analitik dereceli puanlama anahtarı, öz değerlendirme formu, grup değerlendirme formu kullanılarak değerlendirilebilir. Performans görevi olarak öğrencilerden grup etkinliği şeklinde Türkiye nüfusundaki değişim seyrinin nüfusla ilgili fırsat, sorun ve politikalara etkisini belirlemek amacıyla araş-tırma yapmaları ve bu araştırmayı raporlaştırmaları istenebilir. Performans görevi; hazırlık yapma, bilgi toplama, bilgileri çözümleme ve rapor yazma ölçütlerine göre değerlendirilebilir.</t>
-        </is>
-      </c>
+      <c r="C51" s="2" t="n"/>
       <c r="D51" s="2" t="n"/>
       <c r="E51" s="2" t="n"/>
       <c r="F51" s="2" t="n"/>
       <c r="G51" s="2" t="n"/>
       <c r="H51" s="2" t="n"/>
     </row>
-    <row r="52" ht="45.4" customHeight="1">
-      <c r="A52" s="4" t="inlineStr">
-        <is>
-          <t>28-29. haftalar</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="n"/>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>Öğrenme çıktısı; KWL (ne biliyorum-ne bilmek istiyorum-ne öğrendim), performans gö-revi, analitik dereceli puanlama anahtarı, öz değerlendirme formu kullanılarak değerlendirilebilir. Performans görevi olarak öğrencilerden doğal ve beşerî faktörlerin ekonomi üzerindeki etkilerini harita, fotoğraf vb. görsellerle açıklayan bir diyagram hazırlamaları istenebilir. Performans görevi; bilgi toplama, bilgileri düzenleme, görsel materyal kullanma ve diyagram hazırlama ölçütlerine göre değerlendirilebilir.</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="n"/>
-      <c r="E52" s="2" t="n"/>
-      <c r="F52" s="2" t="n"/>
-      <c r="G52" s="2" t="n"/>
-      <c r="H52" s="2" t="n"/>
-    </row>
-    <row r="53" ht="45.4" customHeight="1">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t>30-33. haftalar</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="n"/>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>Öğrenme çıktıları; çalışma yaprağı, yapılandırılmış grid, performans görevi, analitik dere-celi puanlama anahtarı, öz değerlendirme formu kullanılarak değerlendirilebilir. Performans görevi olarak öğrencilerden örnek bir senaryo üzerinden bütüncül afet yönetimine ilişkin önerilerini içeren bir sunum hazırlamaları istenebilir. Performans görevi; bilgi inceleme, içerik, sonuç çıkarma, rapor hazırlama ve sunma ölçütlerine göre değerlendirilebilir.</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="n"/>
-      <c r="E53" s="2" t="n"/>
-      <c r="F53" s="2" t="n"/>
-      <c r="G53" s="2" t="n"/>
-      <c r="H53" s="2" t="n"/>
-    </row>
-    <row r="54" ht="45.4" customHeight="1">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>34. hafta, 35. hafta</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="n"/>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>Öğrenme çıktısı; anlam çözümleme tablosu, açık uçlu sorular, performans görevi, analitik dereceli puanlama anahtarı, öz değerlendirme formu, grup değerlendirme formu kullanılarak değerlendirilebilir. Performans görevi olarak öğrenci gruplarından farklı haritalar üzerinde bölge belirleme kriterlerini dikkate alarak bölgeler oluşturmaları istenebilir. Performans görevi; harita seçme, karşılaştırma yapma, önermede bulunma, sonuç çıkarma, bölge belirleme ve sunma ölçütlerine göre değerlendirilebilir.</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="n"/>
-      <c r="E54" s="2" t="n"/>
-      <c r="F54" s="2" t="n"/>
-      <c r="G54" s="2" t="n"/>
-      <c r="H54" s="2" t="n"/>
-    </row>
-    <row r="56" ht="14" customHeight="1">
-      <c r="A56" s="11" t="inlineStr">
-        <is>
-          <t>SOSYAL - DUYGUSAL ÖĞRENME BECERİLERİ — ünite/hafta bazında</t>
-        </is>
-      </c>
-      <c r="B56" s="12" t="n"/>
-      <c r="C56" s="12" t="n"/>
-      <c r="D56" s="12" t="n"/>
-      <c r="E56" s="12" t="n"/>
-      <c r="F56" s="12" t="n"/>
-      <c r="G56" s="12" t="n"/>
-      <c r="H56" s="12" t="n"/>
-    </row>
-    <row r="57" ht="24.2" customHeight="1">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>1-3. haftalar</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="n"/>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>SDB1.1. Kendini Tanıma (Öz Farkındalık), SDB1.2. Kendini Düzenleme (Öz Düzenleme), SDB1.3. Kendine Uyarlama (Öz Yansıtma), SDB2.1. İletişim, SDB2.2. İş Birliği, SDB2.3. Sos-yal Farkındalık</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="n"/>
-      <c r="E57" s="2" t="n"/>
-      <c r="F57" s="2" t="n"/>
-      <c r="G57" s="2" t="n"/>
-      <c r="H57" s="2" t="n"/>
-    </row>
-    <row r="58" ht="24.2" customHeight="1">
-      <c r="A58" s="4" t="inlineStr">
-        <is>
-          <t>4-8. haftalar, 28-29. haftalar</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="n"/>
-      <c r="C58" s="5" t="inlineStr">
-        <is>
-          <t>SDB1.1. Kendini Tanıma (Öz Farkındalık), SDB1.2. Kendini Düzenleme (Öz Düzenleme), SDB1.3. Kendine Uyarlama (Öz Yansıtma), SDB2.1. İletişim, SDB2.2. İş Birliği</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="n"/>
-      <c r="E58" s="2" t="n"/>
-      <c r="F58" s="2" t="n"/>
-      <c r="G58" s="2" t="n"/>
-      <c r="H58" s="2" t="n"/>
-    </row>
-    <row r="59" ht="45.4" customHeight="1">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t>9. hafta, 10-15. haftalar, 16-17. haftalar, 19. hafta</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="n"/>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>SDB1.1. Kendini Tanıma (Öz Farkındalık), SDB1.2. Kendini Düzenleme (Öz Düzenleme), SDB2.1. İletişim, SDB2.2. İş Birliği, SDB2.3. Sosyal Farkındalık, SDB3.3. Sorumlu Karar Verme</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="n"/>
-      <c r="E59" s="2" t="n"/>
-      <c r="F59" s="2" t="n"/>
-      <c r="G59" s="2" t="n"/>
-      <c r="H59" s="2" t="n"/>
-    </row>
-    <row r="60" ht="34.8" customHeight="1">
-      <c r="A60" s="4" t="inlineStr">
-        <is>
-          <t>20-22. haftalar, 23-26. haftalar, 27. hafta</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="n"/>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>SDB1.1. Kendini Tanıma (Öz Farkındalık), SDB1.2. Kendini Düzenleme (Öz Düzenleme), SDB1.3. Kendine Uyarlama (Öz Yansıtma), SDB2.1. İletişim, SDB2.2. İş Birliği, SDB3.3. Sorumlu Karar Verme</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="n"/>
-      <c r="E60" s="2" t="n"/>
-      <c r="F60" s="2" t="n"/>
-      <c r="G60" s="2" t="n"/>
-      <c r="H60" s="2" t="n"/>
-    </row>
-    <row r="61" ht="24.2" customHeight="1">
-      <c r="A61" s="4" t="inlineStr">
-        <is>
-          <t>30-33. haftalar</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="n"/>
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>DB1.1. Kendini Tanıma (Öz Farkındalık), SDB1.2. Kendini Düzenleme (Öz Düzenleme), SDB1.3. Kendine Uyarlama (Öz Yansıtma), SDB2.1. İletişim, SDB2.2. İş Birliği, SDB2.3. Sos-yal Farkındalık, SDB3.3. Sorumlu Karar Verme</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="n"/>
-      <c r="E61" s="2" t="n"/>
-      <c r="F61" s="2" t="n"/>
-      <c r="G61" s="2" t="n"/>
-      <c r="H61" s="2" t="n"/>
-    </row>
-    <row r="62" ht="24.2" customHeight="1">
-      <c r="A62" s="4" t="inlineStr">
-        <is>
-          <t>34. hafta, 35. hafta</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="n"/>
-      <c r="C62" s="5" t="inlineStr">
-        <is>
-          <t>SDB1.2. Kendini Düzenleme (Öz Düzenleme), SDB1.3. Kendine Uyarlama (Öz Yansıtma), DB2.1. İletişim, SDB2.2. İş Birliği</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="n"/>
-      <c r="E62" s="2" t="n"/>
-      <c r="F62" s="2" t="n"/>
-      <c r="G62" s="2" t="n"/>
-      <c r="H62" s="2" t="n"/>
-    </row>
-    <row r="64" ht="14" customHeight="1">
-      <c r="A64" s="11" t="inlineStr">
-        <is>
-          <t>DEĞERLER — ünite/hafta bazında</t>
-        </is>
-      </c>
-      <c r="B64" s="12" t="n"/>
-      <c r="C64" s="12" t="n"/>
-      <c r="D64" s="12" t="n"/>
-      <c r="E64" s="12" t="n"/>
-      <c r="F64" s="12" t="n"/>
-      <c r="G64" s="12" t="n"/>
-      <c r="H64" s="12" t="n"/>
-    </row>
-    <row r="65" ht="13.6" customHeight="1">
-      <c r="A65" s="4" t="inlineStr">
-        <is>
-          <t>1-3. haftalar</t>
-        </is>
-      </c>
-      <c r="B65" s="2" t="n"/>
-      <c r="C65" s="5" t="inlineStr">
-        <is>
-          <t>D3. Çalışkanlık, D14. Saygı, D16. Sorumluluk, D19. Vatanseverlik</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="n"/>
-      <c r="E65" s="2" t="n"/>
-      <c r="F65" s="2" t="n"/>
-      <c r="G65" s="2" t="n"/>
-      <c r="H65" s="2" t="n"/>
-    </row>
-    <row r="66" ht="13.6" customHeight="1">
-      <c r="A66" s="4" t="inlineStr">
-        <is>
-          <t>4-8. haftalar</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="n"/>
-      <c r="C66" s="5" t="inlineStr">
-        <is>
-          <t>D3. Çalışkanlık, D10. Mütevazılık, D11. Özgürlük, D19. Vatanseverlik</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="n"/>
-      <c r="E66" s="2" t="n"/>
-      <c r="F66" s="2" t="n"/>
-      <c r="G66" s="2" t="n"/>
-      <c r="H66" s="2" t="n"/>
-    </row>
-    <row r="67" ht="45.4" customHeight="1">
-      <c r="A67" s="4" t="inlineStr">
-        <is>
-          <t>9. hafta, 10-15. haftalar, 16-17. haftalar, 19. hafta</t>
-        </is>
-      </c>
-      <c r="B67" s="2" t="n"/>
-      <c r="C67" s="5" t="inlineStr">
-        <is>
-          <t>D3. Çalışkanlık, D5. Duyarlılık, D9. Merhamet, D14. Saygı</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="n"/>
-      <c r="E67" s="2" t="n"/>
-      <c r="F67" s="2" t="n"/>
-      <c r="G67" s="2" t="n"/>
-      <c r="H67" s="2" t="n"/>
-    </row>
-    <row r="68" ht="24.2" customHeight="1">
-      <c r="A68" s="4" t="inlineStr">
-        <is>
-          <t>20-22. haftalar, 23-26. haftalar</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="n"/>
-      <c r="C68" s="5" t="inlineStr">
-        <is>
-          <t>D2. Aile Bütünlüğü, D3. Çalışkanlık, D4. Dostluk, D14. Saygı</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="n"/>
-      <c r="E68" s="2" t="n"/>
-      <c r="F68" s="2" t="n"/>
-      <c r="G68" s="2" t="n"/>
-      <c r="H68" s="2" t="n"/>
-    </row>
-    <row r="69" ht="13.6" customHeight="1">
-      <c r="A69" s="4" t="inlineStr">
-        <is>
-          <t>27. hafta</t>
-        </is>
-      </c>
-      <c r="B69" s="2" t="n"/>
-      <c r="C69" s="5" t="inlineStr">
-        <is>
-          <t>D2. Aile Bütünlüğü, D3. Çalışkanlık, D4. Dostluk, D14. Sayg</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="n"/>
-      <c r="E69" s="2" t="n"/>
-      <c r="F69" s="2" t="n"/>
-      <c r="G69" s="2" t="n"/>
-      <c r="H69" s="2" t="n"/>
-    </row>
-    <row r="70" ht="13.6" customHeight="1">
-      <c r="A70" s="4" t="inlineStr">
-        <is>
-          <t>28-29. haftalar</t>
-        </is>
-      </c>
-      <c r="B70" s="2" t="n"/>
-      <c r="C70" s="5" t="inlineStr">
-        <is>
-          <t>D17. Tasarruf, D19. Vatanseverlik</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="n"/>
-      <c r="E70" s="2" t="n"/>
-      <c r="F70" s="2" t="n"/>
-      <c r="G70" s="2" t="n"/>
-      <c r="H70" s="2" t="n"/>
-    </row>
-    <row r="71" ht="13.6" customHeight="1">
-      <c r="A71" s="4" t="inlineStr">
-        <is>
-          <t>30-33. haftalar</t>
-        </is>
-      </c>
-      <c r="B71" s="2" t="n"/>
-      <c r="C71" s="5" t="inlineStr">
-        <is>
-          <t>D1. Adalet, D5. Duyarlılık, D16. Sorumluluk, D20. Yardımseverlik</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="n"/>
-      <c r="E71" s="2" t="n"/>
-      <c r="F71" s="2" t="n"/>
-      <c r="G71" s="2" t="n"/>
-      <c r="H71" s="2" t="n"/>
-    </row>
-    <row r="72" ht="24.2" customHeight="1">
-      <c r="A72" s="4" t="inlineStr">
-        <is>
-          <t>34. hafta, 35. hafta</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="n"/>
-      <c r="C72" s="5" t="inlineStr">
-        <is>
-          <t>D3. Çalışkanlık</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="n"/>
-      <c r="E72" s="2" t="n"/>
-      <c r="F72" s="2" t="n"/>
-      <c r="G72" s="2" t="n"/>
-      <c r="H72" s="2" t="n"/>
-    </row>
-    <row r="74" ht="14" customHeight="1">
-      <c r="A74" s="11" t="inlineStr">
-        <is>
-          <t>OKURYAZARLIK BECERİLERİ — ünite/hafta bazında</t>
-        </is>
-      </c>
-      <c r="B74" s="12" t="n"/>
-      <c r="C74" s="12" t="n"/>
-      <c r="D74" s="12" t="n"/>
-      <c r="E74" s="12" t="n"/>
-      <c r="F74" s="12" t="n"/>
-      <c r="G74" s="12" t="n"/>
-      <c r="H74" s="12" t="n"/>
-    </row>
-    <row r="75" ht="13.6" customHeight="1">
-      <c r="A75" s="4" t="inlineStr">
-        <is>
-          <t>1-3. haftalar</t>
-        </is>
-      </c>
-      <c r="B75" s="2" t="n"/>
-      <c r="C75" s="5" t="inlineStr">
-        <is>
-          <t>OB1. Bilgi Okuryazarlığı, OB4. Görsel Okuryazarlık</t>
-        </is>
-      </c>
-      <c r="D75" s="2" t="n"/>
-      <c r="E75" s="2" t="n"/>
-      <c r="F75" s="2" t="n"/>
-      <c r="G75" s="2" t="n"/>
-      <c r="H75" s="2" t="n"/>
-    </row>
-    <row r="76" ht="24.2" customHeight="1">
-      <c r="A76" s="4" t="inlineStr">
-        <is>
-          <t>4-8. haftalar, 30-33. haftalar</t>
-        </is>
-      </c>
-      <c r="B76" s="2" t="n"/>
-      <c r="C76" s="5" t="inlineStr">
-        <is>
-          <t>OB1. Bilgi Okuryazarlığı, OB2. Dijital Okuryazarlık, OB4. Görsel Okuryazarlık</t>
-        </is>
-      </c>
-      <c r="D76" s="2" t="n"/>
-      <c r="E76" s="2" t="n"/>
-      <c r="F76" s="2" t="n"/>
-      <c r="G76" s="2" t="n"/>
-      <c r="H76" s="2" t="n"/>
-    </row>
-    <row r="77" ht="45.4" customHeight="1">
-      <c r="A77" s="4" t="inlineStr">
-        <is>
-          <t>9. hafta, 10-15. haftalar, 16-17. haftalar, 19. hafta</t>
-        </is>
-      </c>
-      <c r="B77" s="2" t="n"/>
-      <c r="C77" s="5" t="inlineStr">
-        <is>
-          <t>OB2. Dijital Okuryazarlık, OB4. Görsel Okuryazarlık, OB5. Kültür Okuryazarlığı, OB7. Veri Okuryazarlığı, OB8. Sürdürülebilirlik Okuryazarlığı</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="n"/>
-      <c r="E77" s="2" t="n"/>
-      <c r="F77" s="2" t="n"/>
-      <c r="G77" s="2" t="n"/>
-      <c r="H77" s="2" t="n"/>
-    </row>
-    <row r="78" ht="34.8" customHeight="1">
-      <c r="A78" s="4" t="inlineStr">
-        <is>
-          <t>20-22. haftalar, 23-26. haftalar, 27. hafta</t>
-        </is>
-      </c>
-      <c r="B78" s="2" t="n"/>
-      <c r="C78" s="5" t="inlineStr">
-        <is>
-          <t>OB1. Bilgi Okuryazarlığı, OB4. Görsel Okuryazarlık, OB7. Veri Okuryazarlığı</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="n"/>
-      <c r="E78" s="2" t="n"/>
-      <c r="F78" s="2" t="n"/>
-      <c r="G78" s="2" t="n"/>
-      <c r="H78" s="2" t="n"/>
-    </row>
-    <row r="79" ht="13.6" customHeight="1">
-      <c r="A79" s="4" t="inlineStr">
-        <is>
-          <t>28-29. haftalar</t>
-        </is>
-      </c>
-      <c r="B79" s="2" t="n"/>
-      <c r="C79" s="5" t="inlineStr">
-        <is>
-          <t>OB1. Bilgi Okuryazarlığı</t>
-        </is>
-      </c>
-      <c r="D79" s="2" t="n"/>
-      <c r="E79" s="2" t="n"/>
-      <c r="F79" s="2" t="n"/>
-      <c r="G79" s="2" t="n"/>
-      <c r="H79" s="2" t="n"/>
-    </row>
-    <row r="80" ht="24.2" customHeight="1">
-      <c r="A80" s="4" t="inlineStr">
-        <is>
-          <t>34. hafta, 35. hafta</t>
-        </is>
-      </c>
-      <c r="B80" s="2" t="n"/>
-      <c r="C80" s="5" t="inlineStr">
-        <is>
-          <t>OB2. Dijital Okuryazarlık</t>
-        </is>
-      </c>
-      <c r="D80" s="2" t="n"/>
-      <c r="E80" s="2" t="n"/>
-      <c r="F80" s="2" t="n"/>
-      <c r="G80" s="2" t="n"/>
-      <c r="H80" s="2" t="n"/>
-    </row>
-    <row r="82" ht="14" customHeight="1">
-      <c r="A82" s="11" t="inlineStr">
-        <is>
-          <t>FARKLILAŞTIRMA</t>
-        </is>
-      </c>
-      <c r="B82" s="12" t="n"/>
-      <c r="C82" s="12" t="n"/>
-      <c r="D82" s="12" t="n"/>
-      <c r="E82" s="12" t="n"/>
-      <c r="F82" s="12" t="n"/>
-      <c r="G82" s="12" t="n"/>
-      <c r="H82" s="12" t="n"/>
-    </row>
-    <row r="83" ht="45.4" customHeight="1">
-      <c r="A83" s="5" t="inlineStr">
-        <is>
-          <t>Türkiye Yüzyılı Maarif Modeli Ortak Metni'nde “Farklılaştırılmış öğrenme yaşantılarında öğrencilerin ilgi alanları ile öğrenme profilleri önemlidir ve öğrencilere çeşitli öğrenme yaşantıları sunulur. Farklılaştırma kapsamında yapılacak zenginleştirme ve destekleme uygulamalarında öğrencilerin bireysel farklılıkları (öğrenme hızları, öğrenme stilleri, yetenekleri vb.), ilgi ve ihtiyaçları dikkate alınarak gereken planlamalar yapılır.” ifadesi yer almaktadır. Öğretmenler sınıftaki öğrencilerini gözlemleyerek gerek gördükleri konularda farklılaştırma uygulamalarını ders sürecine dâhil etmelidirler.</t>
-        </is>
-      </c>
-      <c r="B83" s="2" t="n"/>
-      <c r="C83" s="2" t="n"/>
-      <c r="D83" s="2" t="n"/>
-      <c r="E83" s="2" t="n"/>
-      <c r="F83" s="2" t="n"/>
-      <c r="G83" s="2" t="n"/>
-      <c r="H83" s="2" t="n"/>
-    </row>
-    <row r="85" ht="14" customHeight="1">
-      <c r="A85" s="11" t="inlineStr">
-        <is>
-          <t>OKUL TEMELLİ PLANLAMA — ÇERÇEVE PLAN AÇIKLAMASI</t>
-        </is>
-      </c>
-      <c r="B85" s="12" t="n"/>
-      <c r="C85" s="12" t="n"/>
-      <c r="D85" s="12" t="n"/>
-      <c r="E85" s="12" t="n"/>
-      <c r="F85" s="12" t="n"/>
-      <c r="G85" s="12" t="n"/>
-      <c r="H85" s="12" t="n"/>
-    </row>
-    <row r="86" ht="119.6" customHeight="1">
-      <c r="A86" s="5" t="inlineStr">
-        <is>
-          <t>Okul temelli planlama; zümre öğretmenler kurulu tarafından ders kapsamında gerçekleştirilmesi kararlaştırılan araştırma ve gözlem, sosyal etkinlikler, proje çalışmaları, yerel çalışmalar, okuma çalışmaları vb. çalışmaları kapsamaktadır. Çalışmalar için ayrılan süre eğitim-öğretim yılı içinde planlanır ve yıllık planlarda ifade edilir. Bu planlamalar kapsamında yürütülecek öğretim faaliyetleri; öğrenci katılımını desteklemeli, yaparak ve yaşayarak öğrenmeye olanak tanımalı, öğrencinin bütüncül gelişime hizmet etmelidir. *Bu çerçeve planda belirtilen okul temelli planlama haftaları örnek olarak sunulmuştur. Zümre öğretmenler kurulunda aldığınız karara göre okul ve ders koşullarınıza uygun (öğretim programında belirtilen okul temelli planlama ders saati 2 haftadan fazla sürebilir) düzenleyebilirsiniz.Okul temelli planlama; zümre öğretmenler kurulu tarafından ders kapsamında gerçekleştirilmesi kararlaştırılan araştırma ve gözlem, sosyal etkinlikler, proje çalışmaları, yerel çalışmalar, okuma çalışmaları vb. çalışmaları kapsamaktadır. Çalışmalar için ayrılan süre eğitim-öğretim yılı içinde planlanır ve yıllık planlarda ifade edilir. Bu planlamalar kapsamında yürütülecek öğretim faaliyetleri; öğrenci katılımını desteklemeli, yaparak ve yaşayarak öğrenmeye olanak tanımalı, öğrencinin bütüncül gelişime hizmet etmelidir. *Bu çerçeve planda belirtilen okul temelli planlama haftaları örnek olarak sunulmuştur. Zümre öğretmenler kurulunda aldığınız karara göre okul ve ders koşullarınıza uygun (öğretim programında belirtilen okul temelli planlama ders saati 2 haftadan fazla sürebilir) düzenleyebilirsiniz.</t>
-        </is>
-      </c>
-      <c r="B86" s="2" t="n"/>
-      <c r="C86" s="2" t="n"/>
-      <c r="D86" s="2" t="n"/>
-      <c r="E86" s="2" t="n"/>
-      <c r="F86" s="2" t="n"/>
-      <c r="G86" s="2" t="n"/>
-      <c r="H86" s="2" t="n"/>
-    </row>
-    <row r="88" ht="14" customHeight="1">
-      <c r="A88" s="11" t="inlineStr">
-        <is>
-          <t>OKUL UYARLAMA NOTLARI</t>
-        </is>
-      </c>
-      <c r="B88" s="12" t="n"/>
-      <c r="C88" s="12" t="n"/>
-      <c r="D88" s="12" t="n"/>
-      <c r="E88" s="12" t="n"/>
-      <c r="F88" s="12" t="n"/>
-      <c r="G88" s="12" t="n"/>
-      <c r="H88" s="12" t="n"/>
-    </row>
-    <row r="89" ht="24.2" customHeight="1">
-      <c r="A89" s="5" t="inlineStr">
-        <is>
-          <t>GENEL ŞABLON: Bu plan, okulapp.org belge arşivinde yayımlanan genel sürümdür (CC BY 4.0). Köşeli parantezli KIRMIZI alanlar (okul adı, ad-soyad, tarih) okulun bilgileriyle doldurulur; doldurduktan sonra parantez kaldırılır ve yazı rengi siyaha çevrilir.</t>
-        </is>
-      </c>
-      <c r="B89" s="2" t="n"/>
-      <c r="C89" s="2" t="n"/>
-      <c r="D89" s="2" t="n"/>
-      <c r="E89" s="2" t="n"/>
-      <c r="F89" s="2" t="n"/>
-      <c r="G89" s="2" t="n"/>
-      <c r="H89" s="2" t="n"/>
-    </row>
-    <row r="90" ht="34.8" customHeight="1">
-      <c r="A90" s="5" t="inlineStr">
-        <is>
-          <t>KAYNAK: Bu plan, Millî Eğitim Bakanlığının tymm.meb.gov.tr/taslak-cerceve-planlari adresinde yayımladığı 2026-2027 eğitim öğretim yılı Anadolu lisesi coğrafya dersi taslak çerçeve yıllık planının "9.SINIF" sayfasından, içeriği değiştirilmeden A4 yatay sayfaya yeniden yerleştirilerek okula uyarlanmıştır (erişim 29.08.2026). Ünite bazlı öğrenme kanıtları ile programlar arası bileşenler, okunabilirlik için haftalık çizelgenin altındaki bölümlere taşınmıştır.</t>
-        </is>
-      </c>
-      <c r="B90" s="2" t="n"/>
-      <c r="C90" s="2" t="n"/>
-      <c r="D90" s="2" t="n"/>
-      <c r="E90" s="2" t="n"/>
-      <c r="F90" s="2" t="n"/>
-      <c r="G90" s="2" t="n"/>
-      <c r="H90" s="2" t="n"/>
-    </row>
-    <row r="91" ht="45.4" customHeight="1">
-      <c r="A91" s="5" t="inlineStr">
-        <is>
-          <t>ÇALIŞMA TAKVİMİ UYARLAMASI (il millî eğitim müdürlüğü 2026-2027 çalışma takvimi — tarihler Bakanlık takvimiyle ortaktır, ilinizin takvimini kontrol ediniz): Kurban Bayramı tatili 15-19 Mayıs 2027 olup planın 32. haftasına denk gelir; o hafta yalnız perşembe ve cuma günleri ders yapılır ve 19 Mayıs Atatürk'ü Anma, Gençlik ve Spor Bayramı bayram tatili içinde kalır. 28 Ekim 2026 çarşamba yarım gündür; 1 Ocak 2027 cuma ile 23 Nisan 2027 cuma resmî tatildir. Bu günlere gelen ders saatlerinde konu akışı zümre kararıyla yoğunlaştırılarak telafi edilir.</t>
-        </is>
-      </c>
-      <c r="B91" s="2" t="n"/>
-      <c r="C91" s="2" t="n"/>
-      <c r="D91" s="2" t="n"/>
-      <c r="E91" s="2" t="n"/>
-      <c r="F91" s="2" t="n"/>
-      <c r="G91" s="2" t="n"/>
-      <c r="H91" s="2" t="n"/>
-    </row>
-    <row r="92" ht="34.8" customHeight="1">
-      <c r="A92" s="5" t="inlineStr">
-        <is>
-          <t>OKUL TEMELLİ PLANLAMA: Çizelgedeki kırmızı ekler zümre karar taslağıdır; sene başı zümre toplantısında kesinleştirilir, kesinleşen kullanım bu satırlara işlenerek kırmızı ibare siyaha çevrilir. Çerçeve plandaki 18. ve 36. hafta yerleşimi örnektir; zümre kararıyla değiştirilebilir. Öğrenme kanıtları zümre dosyasında toplanır; okul dışına çıkılan çalışmalarda zaman-yer-refakat onayı ile veli izni okulun sosyal etkinlik belgeleri üzerinden alınır.</t>
-        </is>
-      </c>
-      <c r="B92" s="2" t="n"/>
-      <c r="C92" s="2" t="n"/>
-      <c r="D92" s="2" t="n"/>
-      <c r="E92" s="2" t="n"/>
-      <c r="F92" s="2" t="n"/>
-      <c r="G92" s="2" t="n"/>
-      <c r="H92" s="2" t="n"/>
-    </row>
-    <row r="93" ht="13.6" customHeight="1">
-      <c r="A93" s="5" t="inlineStr">
-        <is>
-          <t>ÖLÇME VE DEĞERLENDİRME: Yazılı sınav tarihleri bu planda gösterilmez; okul sınav takvimi ve zümrenin ortak sınav planlamasına göre yürütülür.</t>
-        </is>
-      </c>
-      <c r="B93" s="2" t="n"/>
-      <c r="C93" s="2" t="n"/>
-      <c r="D93" s="2" t="n"/>
-      <c r="E93" s="2" t="n"/>
-      <c r="F93" s="2" t="n"/>
-      <c r="G93" s="2" t="n"/>
-      <c r="H93" s="2" t="n"/>
-    </row>
-    <row r="94" ht="13.6" customHeight="1">
-      <c r="A94" s="5" t="inlineStr">
-        <is>
-          <t>ATATÜRKÇÜLÜK KONULARI: 2488 sayılı Tebliğler Dergisi'ndeki Atatürkçülük konuları, zümre kararı doğrultusunda ilgili ünitelere dağıtılarak işlenir.</t>
-        </is>
-      </c>
-      <c r="B94" s="2" t="n"/>
-      <c r="C94" s="2" t="n"/>
-      <c r="D94" s="2" t="n"/>
-      <c r="E94" s="2" t="n"/>
-      <c r="F94" s="2" t="n"/>
-      <c r="G94" s="2" t="n"/>
-      <c r="H94" s="2" t="n"/>
-    </row>
-    <row r="96" ht="24.2" customHeight="1">
-      <c r="A96" s="5" t="inlineStr">
+    <row r="53" ht="24.2" customHeight="1">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <r>
             <t xml:space="preserve">Bu yıllık plan, Eğitim ve Öğretim Çalışmalarının Planlı Yürütülmesine İlişkin Yönergenin 9 uncu ve 10 uncu maddeleri uyarınca coğrafya zümre öğretmenlerince ortak hazırlanarak okul müdürlüğüne sunulmuştur. Tarih: </t>
@@ -2495,291 +2598,251 @@
           </r>
         </is>
       </c>
-      <c r="B96" s="2" t="n"/>
-      <c r="C96" s="2" t="n"/>
-      <c r="D96" s="2" t="n"/>
-      <c r="E96" s="2" t="n"/>
-      <c r="F96" s="2" t="n"/>
-      <c r="G96" s="2" t="n"/>
-      <c r="H96" s="2" t="n"/>
-    </row>
-    <row r="98" ht="13" customHeight="1">
-      <c r="A98" s="3" t="inlineStr">
+      <c r="B53" s="2" t="n"/>
+      <c r="C53" s="2" t="n"/>
+      <c r="D53" s="2" t="n"/>
+      <c r="E53" s="2" t="n"/>
+      <c r="F53" s="2" t="n"/>
+      <c r="G53" s="2" t="n"/>
+      <c r="H53" s="2" t="n"/>
+    </row>
+    <row r="55" ht="13" customHeight="1">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>Adı Soyadı</t>
         </is>
       </c>
-      <c r="B98" s="12" t="n"/>
-      <c r="C98" s="12" t="n"/>
-      <c r="D98" s="12" t="n"/>
-      <c r="E98" s="3" t="inlineStr">
+      <c r="B55" s="12" t="n"/>
+      <c r="C55" s="12" t="n"/>
+      <c r="D55" s="12" t="n"/>
+      <c r="E55" s="3" t="inlineStr">
         <is>
           <t>Görevi</t>
         </is>
       </c>
-      <c r="F98" s="12" t="n"/>
-      <c r="G98" s="3" t="inlineStr">
+      <c r="F55" s="12" t="n"/>
+      <c r="G55" s="3" t="inlineStr">
         <is>
           <t>İmza</t>
         </is>
       </c>
-      <c r="H98" s="12" t="n"/>
-    </row>
-    <row r="99" ht="22" customHeight="1">
-      <c r="A99" s="13" t="inlineStr">
+      <c r="H55" s="12" t="n"/>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="13" t="inlineStr">
         <is>
           <t>[Adı SOYADI]</t>
         </is>
       </c>
-      <c r="B99" s="2" t="n"/>
-      <c r="C99" s="2" t="n"/>
-      <c r="D99" s="2" t="n"/>
-      <c r="E99" s="4" t="inlineStr">
+      <c r="B56" s="2" t="n"/>
+      <c r="C56" s="2" t="n"/>
+      <c r="D56" s="2" t="n"/>
+      <c r="E56" s="4" t="inlineStr">
         <is>
           <t>Coğrafya Öğretmeni (Zümre Başkanı)</t>
         </is>
       </c>
-      <c r="F99" s="2" t="n"/>
-      <c r="G99" s="5" t="n"/>
-      <c r="H99" s="2" t="n"/>
-    </row>
-    <row r="100" ht="22" customHeight="1">
-      <c r="A100" s="13" t="inlineStr">
+      <c r="F56" s="2" t="n"/>
+      <c r="G56" s="5" t="n"/>
+      <c r="H56" s="2" t="n"/>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="13" t="inlineStr">
         <is>
           <t>[Adı SOYADI]</t>
         </is>
       </c>
-      <c r="B100" s="2" t="n"/>
-      <c r="C100" s="2" t="n"/>
-      <c r="D100" s="2" t="n"/>
-      <c r="E100" s="4" t="inlineStr">
+      <c r="B57" s="2" t="n"/>
+      <c r="C57" s="2" t="n"/>
+      <c r="D57" s="2" t="n"/>
+      <c r="E57" s="4" t="inlineStr">
         <is>
           <t>Coğrafya Öğretmeni</t>
         </is>
       </c>
-      <c r="F100" s="2" t="n"/>
-      <c r="G100" s="5" t="n"/>
-      <c r="H100" s="2" t="n"/>
-    </row>
-    <row r="101" ht="22" customHeight="1">
-      <c r="A101" s="13" t="inlineStr">
+      <c r="F57" s="2" t="n"/>
+      <c r="G57" s="5" t="n"/>
+      <c r="H57" s="2" t="n"/>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="13" t="inlineStr">
         <is>
           <t>[Adı SOYADI]</t>
         </is>
       </c>
-      <c r="B101" s="2" t="n"/>
-      <c r="C101" s="2" t="n"/>
-      <c r="D101" s="2" t="n"/>
-      <c r="E101" s="4" t="inlineStr">
+      <c r="B58" s="2" t="n"/>
+      <c r="C58" s="2" t="n"/>
+      <c r="D58" s="2" t="n"/>
+      <c r="E58" s="4" t="inlineStr">
         <is>
           <t>Coğrafya Öğretmeni</t>
         </is>
       </c>
-      <c r="F101" s="2" t="n"/>
-      <c r="G101" s="5" t="n"/>
-      <c r="H101" s="2" t="n"/>
-    </row>
-    <row r="102" ht="22" customHeight="1">
-      <c r="A102" s="13" t="inlineStr">
+      <c r="F58" s="2" t="n"/>
+      <c r="G58" s="5" t="n"/>
+      <c r="H58" s="2" t="n"/>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="13" t="inlineStr">
         <is>
           <t>[Adı SOYADI]</t>
         </is>
       </c>
-      <c r="B102" s="2" t="n"/>
-      <c r="C102" s="2" t="n"/>
-      <c r="D102" s="2" t="n"/>
-      <c r="E102" s="4" t="inlineStr">
+      <c r="B59" s="2" t="n"/>
+      <c r="C59" s="2" t="n"/>
+      <c r="D59" s="2" t="n"/>
+      <c r="E59" s="4" t="inlineStr">
         <is>
           <t>Coğrafya Öğretmeni</t>
         </is>
       </c>
-      <c r="F102" s="2" t="n"/>
-      <c r="G102" s="5" t="n"/>
-      <c r="H102" s="2" t="n"/>
-    </row>
-    <row r="103" ht="22" customHeight="1">
-      <c r="A103" s="13" t="inlineStr">
+      <c r="F59" s="2" t="n"/>
+      <c r="G59" s="5" t="n"/>
+      <c r="H59" s="2" t="n"/>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="13" t="inlineStr">
         <is>
           <t>[Adı SOYADI]</t>
         </is>
       </c>
-      <c r="B103" s="2" t="n"/>
-      <c r="C103" s="2" t="n"/>
-      <c r="D103" s="2" t="n"/>
-      <c r="E103" s="4" t="inlineStr">
+      <c r="B60" s="2" t="n"/>
+      <c r="C60" s="2" t="n"/>
+      <c r="D60" s="2" t="n"/>
+      <c r="E60" s="4" t="inlineStr">
         <is>
           <t>Coğrafya Öğretmeni</t>
         </is>
       </c>
-      <c r="F103" s="2" t="n"/>
-      <c r="G103" s="5" t="n"/>
-      <c r="H103" s="2" t="n"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="14" t="inlineStr">
+      <c r="F60" s="2" t="n"/>
+      <c r="G60" s="5" t="n"/>
+      <c r="H60" s="2" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="14" t="inlineStr">
         <is>
           <t>UYGUNDUR</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="15" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="15" t="inlineStr">
         <is>
           <t>[../09/2026]</t>
         </is>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" s="16" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="16" t="inlineStr">
         <is>
           <t>[Adı SOYADI]</t>
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" s="17" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="17" t="inlineStr">
         <is>
           <t>Okul Müdürü</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="135">
-    <mergeCell ref="E14:E17"/>
-    <mergeCell ref="A83:H83"/>
-    <mergeCell ref="A51:B51"/>
-    <mergeCell ref="C75:H75"/>
-    <mergeCell ref="A70:B70"/>
-    <mergeCell ref="C59:H59"/>
-    <mergeCell ref="A54:B54"/>
-    <mergeCell ref="C52:H52"/>
-    <mergeCell ref="C61:H61"/>
-    <mergeCell ref="C48:H48"/>
-    <mergeCell ref="C72:H72"/>
-    <mergeCell ref="E99:F99"/>
-    <mergeCell ref="A86:H86"/>
-    <mergeCell ref="G33:G34"/>
-    <mergeCell ref="A76:B76"/>
-    <mergeCell ref="C78:H78"/>
-    <mergeCell ref="F37:F38"/>
-    <mergeCell ref="A99:D99"/>
-    <mergeCell ref="E101:F101"/>
-    <mergeCell ref="A53:B53"/>
-    <mergeCell ref="A62:B62"/>
-    <mergeCell ref="A106:H106"/>
-    <mergeCell ref="E100:F100"/>
-    <mergeCell ref="G100:H100"/>
-    <mergeCell ref="A68:B68"/>
-    <mergeCell ref="A96:H96"/>
-    <mergeCell ref="A101:D101"/>
-    <mergeCell ref="C79:H79"/>
-    <mergeCell ref="G6:G8"/>
-    <mergeCell ref="E102:F102"/>
-    <mergeCell ref="G102:H102"/>
-    <mergeCell ref="A36:A39"/>
-    <mergeCell ref="A48:B48"/>
-    <mergeCell ref="C50:H50"/>
-    <mergeCell ref="A59:B59"/>
-    <mergeCell ref="A107:H107"/>
-    <mergeCell ref="A82:H82"/>
-    <mergeCell ref="A79:B79"/>
-    <mergeCell ref="A61:B61"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="A108:H108"/>
-    <mergeCell ref="D41:H41"/>
-    <mergeCell ref="A27:H27"/>
-    <mergeCell ref="A98:D98"/>
-    <mergeCell ref="A40:A42"/>
-    <mergeCell ref="F6:F8"/>
-    <mergeCell ref="A32:A35"/>
-    <mergeCell ref="C67:H67"/>
-    <mergeCell ref="A23:A26"/>
-    <mergeCell ref="A71:B71"/>
-    <mergeCell ref="A85:H85"/>
-    <mergeCell ref="D6:D10"/>
-    <mergeCell ref="C69:H69"/>
-    <mergeCell ref="A22:H22"/>
-    <mergeCell ref="D14:D17"/>
-    <mergeCell ref="D30:D31"/>
-    <mergeCell ref="C62:H62"/>
-    <mergeCell ref="F14:F17"/>
-    <mergeCell ref="A52:B52"/>
-    <mergeCell ref="A3:A5"/>
-    <mergeCell ref="G99:H99"/>
-    <mergeCell ref="F24:F25"/>
-    <mergeCell ref="A77:B77"/>
-    <mergeCell ref="C54:H54"/>
-    <mergeCell ref="A49:B49"/>
-    <mergeCell ref="A100:D100"/>
+  <mergeCells count="95">
+    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="C9:H9"/>
+    <mergeCell ref="A49:H49"/>
+    <mergeCell ref="C11:H11"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A58:D58"/>
+    <mergeCell ref="G57:H57"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A60:D60"/>
+    <mergeCell ref="A50:H50"/>
+    <mergeCell ref="C32:H32"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="G58:H58"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="C15:H15"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="C24:H24"/>
+    <mergeCell ref="A56:D56"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="C26:H26"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A40:H40"/>
+    <mergeCell ref="G59:H59"/>
+    <mergeCell ref="C10:H10"/>
+    <mergeCell ref="C16:H16"/>
+    <mergeCell ref="E55:F55"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A51:H51"/>
+    <mergeCell ref="C36:H36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A59:D59"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="C19:H19"/>
+    <mergeCell ref="C28:H28"/>
+    <mergeCell ref="C37:H37"/>
+    <mergeCell ref="A42:H42"/>
+    <mergeCell ref="A47:H47"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C6:H6"/>
+    <mergeCell ref="A62:H62"/>
+    <mergeCell ref="C14:H14"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C4:H4"/>
+    <mergeCell ref="G60:H60"/>
+    <mergeCell ref="E58:F58"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A48:H48"/>
     <mergeCell ref="A64:H64"/>
-    <mergeCell ref="D24:D26"/>
-    <mergeCell ref="A69:B69"/>
-    <mergeCell ref="A88:H88"/>
-    <mergeCell ref="A102:D102"/>
-    <mergeCell ref="A78:B78"/>
-    <mergeCell ref="D21:H21"/>
-    <mergeCell ref="C71:H71"/>
-    <mergeCell ref="A65:B65"/>
-    <mergeCell ref="G101:H101"/>
-    <mergeCell ref="C76:H76"/>
-    <mergeCell ref="E103:F103"/>
-    <mergeCell ref="A75:B75"/>
-    <mergeCell ref="G103:H103"/>
-    <mergeCell ref="A90:H90"/>
-    <mergeCell ref="G37:G38"/>
-    <mergeCell ref="A80:B80"/>
-    <mergeCell ref="G24:G25"/>
-    <mergeCell ref="D28:D29"/>
-    <mergeCell ref="A74:H74"/>
-    <mergeCell ref="A56:H56"/>
-    <mergeCell ref="A103:D103"/>
-    <mergeCell ref="G14:G17"/>
-    <mergeCell ref="C57:H57"/>
-    <mergeCell ref="C66:H66"/>
-    <mergeCell ref="A57:B57"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="C53:H53"/>
-    <mergeCell ref="C68:H68"/>
-    <mergeCell ref="C58:H58"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="A28:A31"/>
-    <mergeCell ref="A15:A18"/>
-    <mergeCell ref="A67:B67"/>
-    <mergeCell ref="C65:H65"/>
-    <mergeCell ref="C47:H47"/>
-    <mergeCell ref="A92:H92"/>
-    <mergeCell ref="A60:B60"/>
-    <mergeCell ref="E98:F98"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="C80:H80"/>
-    <mergeCell ref="G98:H98"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="C27:H27"/>
+    <mergeCell ref="C8:H8"/>
+    <mergeCell ref="C17:H17"/>
+    <mergeCell ref="E59:F59"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="C34:H34"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="E57:F57"/>
+    <mergeCell ref="A53:H53"/>
+    <mergeCell ref="C5:H5"/>
+    <mergeCell ref="A63:H63"/>
+    <mergeCell ref="A57:D57"/>
+    <mergeCell ref="E56:F56"/>
+    <mergeCell ref="C29:H29"/>
+    <mergeCell ref="G56:H56"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A39:H39"/>
+    <mergeCell ref="C22:H22"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A94:H94"/>
-    <mergeCell ref="C51:H51"/>
-    <mergeCell ref="C60:H60"/>
-    <mergeCell ref="C70:H70"/>
-    <mergeCell ref="A19:A21"/>
-    <mergeCell ref="A66:B66"/>
+    <mergeCell ref="A45:H45"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A65:H65"/>
+    <mergeCell ref="C23:H23"/>
+    <mergeCell ref="A18:B18"/>
     <mergeCell ref="A46:H46"/>
-    <mergeCell ref="A89:H89"/>
-    <mergeCell ref="A50:B50"/>
-    <mergeCell ref="A12:H12"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="A105:H105"/>
-    <mergeCell ref="A47:B47"/>
-    <mergeCell ref="C49:H49"/>
-    <mergeCell ref="C77:H77"/>
-    <mergeCell ref="E6:E8"/>
-    <mergeCell ref="A6:A10"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="A72:B72"/>
-    <mergeCell ref="A91:H91"/>
-    <mergeCell ref="D35:D38"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="D3:D5"/>
-    <mergeCell ref="A93:H93"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="A58:B58"/>
+    <mergeCell ref="E60:F60"/>
+    <mergeCell ref="C7:H7"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="C18:H18"/>
+    <mergeCell ref="G55:H55"/>
+    <mergeCell ref="C33:H33"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A43:H43"/>
+    <mergeCell ref="A55:D55"/>
+    <mergeCell ref="C35:H35"/>
   </mergeCells>
   <pageMargins left="0.39" right="0.39" top="0.55" bottom="0.55" header="0.25" footer="0.25"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Belge arşivi: coğrafya yıllık planları 2026.08.2 — MEB kaynağındaki çift yapıştırılmış okul temelli planlama açıklaması tekilleştirildi
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/evrak/cografya-yillik-planlari/GNL-CYP-CP-001_Cografya_9_Sinif_Yillik_Plani_v1.0.xlsx
+++ b/public/evrak/cografya-yillik-planlari/GNL-CYP-CP-001_Cografya_9_Sinif_Yillik_Plani_v1.0.xlsx
@@ -2470,10 +2470,10 @@
       <c r="G42" s="12" t="n"/>
       <c r="H42" s="12" t="n"/>
     </row>
-    <row r="43" ht="119.6" customHeight="1">
+    <row r="43" ht="66.59999999999999" customHeight="1">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>Okul temelli planlama; zümre öğretmenler kurulu tarafından ders kapsamında gerçekleştirilmesi kararlaştırılan araştırma ve gözlem, sosyal etkinlikler, proje çalışmaları, yerel çalışmalar, okuma çalışmaları vb. çalışmaları kapsamaktadır. Çalışmalar için ayrılan süre eğitim-öğretim yılı içinde planlanır ve yıllık planlarda ifade edilir. Bu planlamalar kapsamında yürütülecek öğretim faaliyetleri; öğrenci katılımını desteklemeli, yaparak ve yaşayarak öğrenmeye olanak tanımalı, öğrencinin bütüncül gelişime hizmet etmelidir. *Bu çerçeve planda belirtilen okul temelli planlama haftaları örnek olarak sunulmuştur. Zümre öğretmenler kurulunda aldığınız karara göre okul ve ders koşullarınıza uygun (öğretim programında belirtilen okul temelli planlama ders saati 2 haftadan fazla sürebilir) düzenleyebilirsiniz.Okul temelli planlama; zümre öğretmenler kurulu tarafından ders kapsamında gerçekleştirilmesi kararlaştırılan araştırma ve gözlem, sosyal etkinlikler, proje çalışmaları, yerel çalışmalar, okuma çalışmaları vb. çalışmaları kapsamaktadır. Çalışmalar için ayrılan süre eğitim-öğretim yılı içinde planlanır ve yıllık planlarda ifade edilir. Bu planlamalar kapsamında yürütülecek öğretim faaliyetleri; öğrenci katılımını desteklemeli, yaparak ve yaşayarak öğrenmeye olanak tanımalı, öğrencinin bütüncül gelişime hizmet etmelidir. *Bu çerçeve planda belirtilen okul temelli planlama haftaları örnek olarak sunulmuştur. Zümre öğretmenler kurulunda aldığınız karara göre okul ve ders koşullarınıza uygun (öğretim programında belirtilen okul temelli planlama ders saati 2 haftadan fazla sürebilir) düzenleyebilirsiniz.</t>
+          <t>Okul temelli planlama; zümre öğretmenler kurulu tarafından ders kapsamında gerçekleştirilmesi kararlaştırılan araştırma ve gözlem, sosyal etkinlikler, proje çalışmaları, yerel çalışmalar, okuma çalışmaları vb. çalışmaları kapsamaktadır. Çalışmalar için ayrılan süre eğitim-öğretim yılı içinde planlanır ve yıllık planlarda ifade edilir. Bu planlamalar kapsamında yürütülecek öğretim faaliyetleri; öğrenci katılımını desteklemeli, yaparak ve yaşayarak öğrenmeye olanak tanımalı, öğrencinin bütüncül gelişime hizmet etmelidir. *Bu çerçeve planda belirtilen okul temelli planlama haftaları örnek olarak sunulmuştur. Zümre öğretmenler kurulunda aldığınız karara göre okul ve ders koşullarınıza uygun (öğretim programında belirtilen okul temelli planlama ders saati 2 haftadan fazla sürebilir) düzenleyebilirsiniz.</t>
         </is>
       </c>
       <c r="B43" s="2" t="n"/>

</xml_diff>

<commit_message>
Belge arşivi: coğrafya yıllık planları 2026.08.3 — çizelge sonundaki içeriksiz kenarlıklı satırlar kaldırıldı
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/evrak/cografya-yillik-planlari/GNL-CYP-CP-001_Cografya_9_Sinif_Yillik_Plani_v1.0.xlsx
+++ b/public/evrak/cografya-yillik-planlari/GNL-CYP-CP-001_Cografya_9_Sinif_Yillik_Plani_v1.0.xlsx
@@ -545,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.3" customWidth="1" min="1" max="1"/>
@@ -1746,26 +1746,6 @@
       <c r="F42" s="9" t="n"/>
       <c r="G42" s="9" t="n"/>
       <c r="H42" s="9" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="n"/>
-      <c r="B43" s="5" t="n"/>
-      <c r="C43" s="5" t="n"/>
-      <c r="D43" s="5" t="n"/>
-      <c r="E43" s="5" t="n"/>
-      <c r="F43" s="5" t="n"/>
-      <c r="G43" s="5" t="n"/>
-      <c r="H43" s="5" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="n"/>
-      <c r="B44" s="5" t="n"/>
-      <c r="C44" s="5" t="n"/>
-      <c r="D44" s="5" t="n"/>
-      <c r="E44" s="5" t="n"/>
-      <c r="F44" s="5" t="n"/>
-      <c r="G44" s="5" t="n"/>
-      <c r="H44" s="5" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="41">

</xml_diff>